<commit_message>
Update agriculture 5.xlsx with new data
</commit_message>
<xml_diff>
--- a/agriculture 5.xlsx
+++ b/agriculture 5.xlsx
@@ -288,7 +288,6 @@
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
         <family val="2"/>
-        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Description</t>
     </r>
@@ -298,7 +297,6 @@
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
         <family val="2"/>
-        <charset val="1"/>
       </rPr>
       <t xml:space="preserve"> : Directorate of Economics and Statistics, Dept. of Agriculture, Cooperation and Farmers Welfare, Ministry of Agriculture, Govt. of India</t>
     </r>
@@ -312,7 +310,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -343,11 +341,22 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -358,7 +367,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="3">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -368,13 +377,6 @@
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="thin"/>
-      <right/>
-      <top style="thin"/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left/>
       <right/>
       <top style="thin"/>
       <bottom/>
@@ -438,20 +440,20 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -476,7 +478,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E1048576"/>
-  <sheetFormatPr defaultColWidth="10.8125" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.82421875" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="23.54"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24.8"/>
@@ -1500,51 +1502,51 @@
       <c r="C74" s="5"/>
       <c r="D74" s="5"/>
     </row>
-    <row r="75" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B75" s="7"/>
-      <c r="C75" s="7"/>
-      <c r="D75" s="7"/>
+      <c r="B75" s="6"/>
+      <c r="C75" s="6"/>
+      <c r="D75" s="6"/>
     </row>
     <row r="76" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A76" s="8" t="s">
+      <c r="A76" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="B76" s="8"/>
-      <c r="C76" s="8"/>
-      <c r="D76" s="8"/>
+      <c r="B76" s="7"/>
+      <c r="C76" s="7"/>
+      <c r="D76" s="7"/>
     </row>
     <row r="77" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A77" s="8"/>
-      <c r="B77" s="8"/>
-      <c r="C77" s="8"/>
-      <c r="D77" s="8"/>
+      <c r="A77" s="7"/>
+      <c r="B77" s="7"/>
+      <c r="C77" s="7"/>
+      <c r="D77" s="7"/>
     </row>
     <row r="78" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A78" s="9" t="s">
+      <c r="A78" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="B78" s="9"/>
-      <c r="C78" s="9"/>
-      <c r="D78" s="9"/>
+      <c r="B78" s="8"/>
+      <c r="C78" s="8"/>
+      <c r="D78" s="8"/>
     </row>
     <row r="79" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A79" s="9"/>
-      <c r="B79" s="9"/>
-      <c r="C79" s="9"/>
-      <c r="D79" s="9"/>
+      <c r="A79" s="8"/>
+      <c r="B79" s="8"/>
+      <c r="C79" s="8"/>
+      <c r="D79" s="8"/>
     </row>
     <row r="80" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A80" s="10" t="s">
+      <c r="A80" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="B80" s="10"/>
-      <c r="C80" s="10"/>
-      <c r="D80" s="10"/>
-    </row>
-    <row r="81" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B80" s="9"/>
+      <c r="C80" s="9"/>
+      <c r="D80" s="9"/>
+    </row>
+    <row r="81" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="10"/>
       <c r="B81" s="10"/>
       <c r="C81" s="10"/>
@@ -1553,11 +1555,12 @@
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A74:D74"/>
+    <mergeCell ref="A75:D75"/>
     <mergeCell ref="A76:D77"/>
     <mergeCell ref="A78:D79"/>
-    <mergeCell ref="A80:D81"/>
+    <mergeCell ref="A80:D80"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>